<commit_message>
#1 Changes Completed and Deliverables Generated
</commit_message>
<xml_diff>
--- a/Design Files/Gear_Trak-v1.0/Deliverables/BOM/Client-BOM-Gear_Trak-v1.0.xlsx
+++ b/Design Files/Gear_Trak-v1.0/Deliverables/BOM/Client-BOM-Gear_Trak-v1.0.xlsx
@@ -1,25 +1,26 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
-  <fileVersion appName="xl" lastEdited="6" lowestEdited="6" rupBuild="14420"/>
-  <workbookPr codeName="ThisWorkbook" defaultThemeVersion="153222"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="20417"/>
+  <workbookPr codeName="ThisWorkbook"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\eSpark-Consultants\stephen-geartrak\Design Files\Gear_Trak-v1.0\Deliverables\BOM\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\eSpark-Consultants\GitHub\stephen-geartrak\Design Files\Gear_Trak-v1.0\Deliverables\BOM\"/>
     </mc:Choice>
   </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{79C0BF86-FC0B-4302-B311-E4ABAE29C0BD}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15840"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="162913"/>
+  <calcPr calcId="191029"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="623" uniqueCount="422">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="622" uniqueCount="420">
   <si>
     <t>#</t>
   </si>
@@ -420,9 +421,6 @@
     <t>1.0mm pitch connector side entry SMD</t>
   </si>
   <si>
-    <t>5A 1 16P Female Type-C SMD USB Connectors ROHS</t>
-  </si>
-  <si>
     <t>NanoSIM SMD SIM Card Connectors</t>
   </si>
   <si>
@@ -462,9 +460,6 @@
     <t>RED LED 0603 Light Emitting Diodes</t>
   </si>
   <si>
-    <t>Pin Header 2x5, 1.27mm (50mil)</t>
-  </si>
-  <si>
     <t>30V 5.8A 35mΩ@10V,5.8A 350mW N Channel SOT-23 MOSFETs ROHS</t>
   </si>
   <si>
@@ -612,9 +607,6 @@
     <t>CONN_SMD_3P_1mm_SM03B-SRSS-TB</t>
   </si>
   <si>
-    <t>TYPE-C-31-M-12_</t>
-  </si>
-  <si>
     <t>XUNPU_SMN-303</t>
   </si>
   <si>
@@ -651,9 +643,6 @@
     <t>LED-0603</t>
   </si>
   <si>
-    <t>Header_SMT_2X5-1.27mm</t>
-  </si>
-  <si>
     <t>SOT-23a</t>
   </si>
   <si>
@@ -771,9 +760,6 @@
     <t>BLM21PG221SN1D</t>
   </si>
   <si>
-    <t>TYPE-C-31-M-12</t>
-  </si>
-  <si>
     <t>SMN-303</t>
   </si>
   <si>
@@ -798,9 +784,6 @@
     <t>NCD0603R3</t>
   </si>
   <si>
-    <t>1325B-1205S0Z080CR02</t>
-  </si>
-  <si>
     <t>RC0201JR-070RL</t>
   </si>
   <si>
@@ -918,9 +901,6 @@
     <t>Foshan NationStar Optoelectronics</t>
   </si>
   <si>
-    <t>W-CON</t>
-  </si>
-  <si>
     <t>KOA Speer</t>
   </si>
   <si>
@@ -1092,9 +1072,6 @@
     <t>RED</t>
   </si>
   <si>
-    <t>PROG</t>
-  </si>
-  <si>
     <t>AO3400</t>
   </si>
   <si>
@@ -1285,12 +1262,30 @@
   </si>
   <si>
     <t>Ignion</t>
+  </si>
+  <si>
+    <t>USB C RECEPTACLE, 16PIN</t>
+  </si>
+  <si>
+    <t>203615-0003</t>
+  </si>
+  <si>
+    <t>Molex</t>
+  </si>
+  <si>
+    <t>CONN RCPT 10POS 0.05 GOLD SMD</t>
+  </si>
+  <si>
+    <t>20021321-00010C4LF</t>
+  </si>
+  <si>
+    <t>Amphenol Communications Solutions</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <fonts count="8" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
@@ -1504,9 +1499,6 @@
     <xf numFmtId="0" fontId="5" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="6" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -1515,6 +1507,9 @@
     </xf>
     <xf numFmtId="0" fontId="7" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1801,7 +1796,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <sheetPr codeName="Sheet1"/>
   <dimension ref="A1:K90"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -1827,9 +1822,9 @@
       <c r="F1" s="2"/>
       <c r="G1" s="2"/>
       <c r="H1" s="2"/>
-      <c r="I1" s="14"/>
-      <c r="J1" s="14"/>
-      <c r="K1" s="14"/>
+      <c r="I1" s="17"/>
+      <c r="J1" s="17"/>
+      <c r="K1" s="17"/>
     </row>
     <row r="2" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A2" s="1"/>
@@ -1846,22 +1841,22 @@
         <v>104</v>
       </c>
       <c r="F2" s="5" t="s">
-        <v>179</v>
+        <v>177</v>
       </c>
       <c r="G2" s="6" t="s">
-        <v>231</v>
+        <v>227</v>
       </c>
       <c r="H2" s="5" t="s">
-        <v>285</v>
+        <v>279</v>
       </c>
       <c r="I2" s="6" t="s">
-        <v>379</v>
+        <v>371</v>
       </c>
       <c r="J2" s="5" t="s">
-        <v>378</v>
+        <v>370</v>
       </c>
       <c r="K2" s="5" t="s">
-        <v>380</v>
+        <v>372</v>
       </c>
     </row>
     <row r="3" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
@@ -1880,16 +1875,16 @@
         <v>105</v>
       </c>
       <c r="F3" s="7" t="s">
-        <v>180</v>
+        <v>178</v>
       </c>
       <c r="G3" s="8" t="s">
-        <v>232</v>
+        <v>228</v>
       </c>
       <c r="H3" s="7" t="s">
-        <v>286</v>
+        <v>280</v>
       </c>
       <c r="I3" s="8" t="s">
-        <v>312</v>
+        <v>305</v>
       </c>
       <c r="J3" s="7">
         <v>1</v>
@@ -1912,16 +1907,16 @@
         <v>106</v>
       </c>
       <c r="F4" s="9" t="s">
-        <v>181</v>
+        <v>179</v>
       </c>
       <c r="G4" s="10" t="s">
-        <v>181</v>
+        <v>179</v>
       </c>
       <c r="H4" s="9" t="s">
-        <v>287</v>
+        <v>281</v>
       </c>
       <c r="I4" s="10" t="s">
-        <v>181</v>
+        <v>179</v>
       </c>
       <c r="J4" s="9">
         <v>1</v>
@@ -1942,16 +1937,16 @@
       </c>
       <c r="E5" s="8"/>
       <c r="F5" s="7" t="s">
-        <v>182</v>
+        <v>180</v>
       </c>
       <c r="G5" s="8" t="s">
-        <v>313</v>
+        <v>306</v>
       </c>
       <c r="H5" s="7" t="s">
-        <v>421</v>
+        <v>413</v>
       </c>
       <c r="I5" s="8" t="s">
-        <v>313</v>
+        <v>306</v>
       </c>
       <c r="J5" s="7">
         <v>1</v>
@@ -1974,16 +1969,16 @@
         <v>107</v>
       </c>
       <c r="F6" s="9" t="s">
-        <v>183</v>
+        <v>181</v>
       </c>
       <c r="G6" s="10" t="s">
-        <v>389</v>
+        <v>381</v>
       </c>
       <c r="H6" s="9" t="s">
-        <v>390</v>
+        <v>382</v>
       </c>
       <c r="I6" s="10" t="s">
-        <v>314</v>
+        <v>307</v>
       </c>
       <c r="J6" s="9">
         <v>1</v>
@@ -2006,16 +2001,16 @@
         <v>108</v>
       </c>
       <c r="F7" s="7" t="s">
-        <v>184</v>
+        <v>182</v>
       </c>
       <c r="G7" s="8" t="s">
-        <v>391</v>
+        <v>383</v>
       </c>
       <c r="H7" s="9" t="s">
-        <v>390</v>
+        <v>382</v>
       </c>
       <c r="I7" s="8" t="s">
-        <v>315</v>
+        <v>308</v>
       </c>
       <c r="J7" s="7">
         <v>1</v>
@@ -2038,16 +2033,16 @@
         <v>108</v>
       </c>
       <c r="F8" s="9" t="s">
-        <v>184</v>
+        <v>182</v>
       </c>
       <c r="G8" s="10" t="s">
-        <v>392</v>
+        <v>384</v>
       </c>
       <c r="H8" s="9" t="s">
-        <v>390</v>
+        <v>382</v>
       </c>
       <c r="I8" s="10" t="s">
-        <v>316</v>
+        <v>309</v>
       </c>
       <c r="J8" s="9">
         <v>1</v>
@@ -2070,16 +2065,16 @@
         <v>108</v>
       </c>
       <c r="F9" s="7" t="s">
-        <v>184</v>
+        <v>182</v>
       </c>
       <c r="G9" s="8" t="s">
-        <v>393</v>
+        <v>385</v>
       </c>
       <c r="H9" s="9" t="s">
-        <v>390</v>
+        <v>382</v>
       </c>
       <c r="I9" s="8" t="s">
-        <v>317</v>
+        <v>310</v>
       </c>
       <c r="J9" s="7">
         <v>1</v>
@@ -2102,16 +2097,16 @@
         <v>109</v>
       </c>
       <c r="F10" s="9" t="s">
-        <v>183</v>
+        <v>181</v>
       </c>
       <c r="G10" s="10" t="s">
-        <v>394</v>
+        <v>386</v>
       </c>
       <c r="H10" s="9" t="s">
-        <v>390</v>
+        <v>382</v>
       </c>
       <c r="I10" s="10" t="s">
-        <v>318</v>
+        <v>311</v>
       </c>
       <c r="J10" s="9">
         <v>2</v>
@@ -2134,16 +2129,16 @@
         <v>108</v>
       </c>
       <c r="F11" s="7" t="s">
-        <v>184</v>
+        <v>182</v>
       </c>
       <c r="G11" s="8" t="s">
-        <v>395</v>
+        <v>387</v>
       </c>
       <c r="H11" s="9" t="s">
-        <v>390</v>
+        <v>382</v>
       </c>
       <c r="I11" s="8" t="s">
-        <v>319</v>
+        <v>312</v>
       </c>
       <c r="J11" s="7">
         <v>1</v>
@@ -2166,16 +2161,16 @@
         <v>109</v>
       </c>
       <c r="F12" s="9" t="s">
-        <v>183</v>
+        <v>181</v>
       </c>
       <c r="G12" s="10" t="s">
-        <v>396</v>
+        <v>388</v>
       </c>
       <c r="H12" s="9" t="s">
-        <v>390</v>
+        <v>382</v>
       </c>
       <c r="I12" s="10" t="s">
-        <v>320</v>
+        <v>313</v>
       </c>
       <c r="J12" s="9">
         <v>1</v>
@@ -2198,16 +2193,16 @@
         <v>109</v>
       </c>
       <c r="F13" s="7" t="s">
-        <v>183</v>
+        <v>181</v>
       </c>
       <c r="G13" s="8" t="s">
-        <v>397</v>
+        <v>389</v>
       </c>
       <c r="H13" s="9" t="s">
-        <v>390</v>
+        <v>382</v>
       </c>
       <c r="I13" s="8" t="s">
-        <v>321</v>
+        <v>314</v>
       </c>
       <c r="J13" s="7">
         <v>1</v>
@@ -2230,16 +2225,16 @@
         <v>110</v>
       </c>
       <c r="F14" s="9" t="s">
-        <v>185</v>
+        <v>183</v>
       </c>
       <c r="G14" s="10" t="s">
-        <v>233</v>
+        <v>229</v>
       </c>
       <c r="H14" s="9" t="s">
-        <v>288</v>
+        <v>282</v>
       </c>
       <c r="I14" s="10" t="s">
-        <v>322</v>
+        <v>315</v>
       </c>
       <c r="J14" s="9">
         <v>3</v>
@@ -2262,16 +2257,16 @@
         <v>109</v>
       </c>
       <c r="F15" s="7" t="s">
-        <v>183</v>
+        <v>181</v>
       </c>
       <c r="G15" s="8" t="s">
-        <v>398</v>
+        <v>390</v>
       </c>
       <c r="H15" s="7" t="s">
-        <v>399</v>
+        <v>391</v>
       </c>
       <c r="I15" s="8" t="s">
-        <v>323</v>
+        <v>316</v>
       </c>
       <c r="J15" s="7">
         <v>1</v>
@@ -2294,16 +2289,16 @@
         <v>111</v>
       </c>
       <c r="F16" s="9" t="s">
-        <v>185</v>
+        <v>183</v>
       </c>
       <c r="G16" s="10" t="s">
-        <v>234</v>
+        <v>230</v>
       </c>
       <c r="H16" s="9" t="s">
-        <v>288</v>
+        <v>282</v>
       </c>
       <c r="I16" s="10" t="s">
-        <v>324</v>
+        <v>317</v>
       </c>
       <c r="J16" s="9">
         <v>2</v>
@@ -2326,16 +2321,16 @@
         <v>112</v>
       </c>
       <c r="F17" s="7" t="s">
-        <v>186</v>
+        <v>184</v>
       </c>
       <c r="G17" s="8" t="s">
-        <v>235</v>
+        <v>231</v>
       </c>
       <c r="H17" s="7" t="s">
-        <v>289</v>
+        <v>283</v>
       </c>
       <c r="I17" s="8" t="s">
-        <v>325</v>
+        <v>318</v>
       </c>
       <c r="J17" s="7">
         <v>15</v>
@@ -2358,16 +2353,16 @@
         <v>113</v>
       </c>
       <c r="F18" s="9" t="s">
-        <v>187</v>
+        <v>185</v>
       </c>
       <c r="G18" s="10" t="s">
-        <v>400</v>
+        <v>392</v>
       </c>
       <c r="H18" s="9" t="s">
-        <v>390</v>
+        <v>382</v>
       </c>
       <c r="I18" s="10" t="s">
-        <v>326</v>
+        <v>319</v>
       </c>
       <c r="J18" s="9">
         <v>2</v>
@@ -2390,16 +2385,16 @@
         <v>114</v>
       </c>
       <c r="F19" s="7" t="s">
-        <v>185</v>
+        <v>183</v>
       </c>
       <c r="G19" s="8" t="s">
-        <v>236</v>
+        <v>232</v>
       </c>
       <c r="H19" s="7" t="s">
-        <v>290</v>
+        <v>284</v>
       </c>
       <c r="I19" s="8" t="s">
-        <v>327</v>
+        <v>320</v>
       </c>
       <c r="J19" s="7">
         <v>5</v>
@@ -2422,16 +2417,16 @@
         <v>108</v>
       </c>
       <c r="F20" s="9" t="s">
-        <v>184</v>
+        <v>182</v>
       </c>
       <c r="G20" s="10" t="s">
-        <v>237</v>
+        <v>233</v>
       </c>
       <c r="H20" s="9" t="s">
-        <v>291</v>
+        <v>285</v>
       </c>
       <c r="I20" s="10" t="s">
-        <v>328</v>
+        <v>321</v>
       </c>
       <c r="J20" s="9">
         <v>1</v>
@@ -2454,16 +2449,16 @@
         <v>115</v>
       </c>
       <c r="F21" s="7" t="s">
-        <v>185</v>
+        <v>183</v>
       </c>
       <c r="G21" s="8" t="s">
-        <v>238</v>
+        <v>234</v>
       </c>
       <c r="H21" s="7" t="s">
-        <v>291</v>
+        <v>285</v>
       </c>
       <c r="I21" s="8" t="s">
-        <v>329</v>
+        <v>322</v>
       </c>
       <c r="J21" s="7">
         <v>4</v>
@@ -2486,16 +2481,16 @@
         <v>116</v>
       </c>
       <c r="F22" s="9" t="s">
-        <v>185</v>
+        <v>183</v>
       </c>
       <c r="G22" s="10" t="s">
-        <v>239</v>
+        <v>235</v>
       </c>
       <c r="H22" s="9" t="s">
-        <v>291</v>
+        <v>285</v>
       </c>
       <c r="I22" s="10" t="s">
-        <v>330</v>
+        <v>323</v>
       </c>
       <c r="J22" s="9">
         <v>2</v>
@@ -2518,16 +2513,16 @@
         <v>117</v>
       </c>
       <c r="F23" s="7" t="s">
-        <v>185</v>
+        <v>183</v>
       </c>
       <c r="G23" s="8" t="s">
-        <v>240</v>
+        <v>236</v>
       </c>
       <c r="H23" s="7" t="s">
-        <v>288</v>
+        <v>282</v>
       </c>
       <c r="I23" s="8" t="s">
-        <v>331</v>
+        <v>324</v>
       </c>
       <c r="J23" s="7">
         <v>1</v>
@@ -2550,16 +2545,16 @@
         <v>118</v>
       </c>
       <c r="F24" s="9" t="s">
-        <v>185</v>
+        <v>183</v>
       </c>
       <c r="G24" s="10" t="s">
-        <v>241</v>
+        <v>237</v>
       </c>
       <c r="H24" s="9" t="s">
-        <v>288</v>
+        <v>282</v>
       </c>
       <c r="I24" s="10" t="s">
-        <v>332</v>
+        <v>325</v>
       </c>
       <c r="J24" s="9">
         <v>1</v>
@@ -2575,29 +2570,29 @@
       <c r="C25" s="12" t="s">
         <v>3</v>
       </c>
-      <c r="D25" s="15" t="s">
+      <c r="D25" s="14" t="s">
         <v>38</v>
       </c>
-      <c r="E25" s="16" t="s">
+      <c r="E25" s="15" t="s">
         <v>119</v>
       </c>
-      <c r="F25" s="15" t="s">
-        <v>184</v>
-      </c>
-      <c r="G25" s="16" t="s">
-        <v>401</v>
-      </c>
-      <c r="H25" s="15" t="s">
-        <v>401</v>
-      </c>
-      <c r="I25" s="16" t="s">
-        <v>333</v>
-      </c>
-      <c r="J25" s="15">
+      <c r="F25" s="14" t="s">
+        <v>182</v>
+      </c>
+      <c r="G25" s="15" t="s">
+        <v>393</v>
+      </c>
+      <c r="H25" s="14" t="s">
+        <v>393</v>
+      </c>
+      <c r="I25" s="15" t="s">
+        <v>326</v>
+      </c>
+      <c r="J25" s="14">
         <v>2</v>
       </c>
-      <c r="K25" s="17" t="s">
-        <v>381</v>
+      <c r="K25" s="16" t="s">
+        <v>373</v>
       </c>
     </row>
     <row r="26" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
@@ -2616,16 +2611,16 @@
         <v>120</v>
       </c>
       <c r="F26" s="9" t="s">
-        <v>185</v>
+        <v>183</v>
       </c>
       <c r="G26" s="10" t="s">
-        <v>242</v>
+        <v>238</v>
       </c>
       <c r="H26" s="9" t="s">
-        <v>291</v>
+        <v>285</v>
       </c>
       <c r="I26" s="10" t="s">
-        <v>334</v>
+        <v>327</v>
       </c>
       <c r="J26" s="9">
         <v>1</v>
@@ -2648,16 +2643,16 @@
         <v>121</v>
       </c>
       <c r="F27" s="7" t="s">
-        <v>185</v>
+        <v>183</v>
       </c>
       <c r="G27" s="8" t="s">
-        <v>243</v>
+        <v>239</v>
       </c>
       <c r="H27" s="7" t="s">
-        <v>291</v>
+        <v>285</v>
       </c>
       <c r="I27" s="8" t="s">
-        <v>335</v>
+        <v>328</v>
       </c>
       <c r="J27" s="7">
         <v>9</v>
@@ -2680,16 +2675,16 @@
         <v>122</v>
       </c>
       <c r="F28" s="9" t="s">
-        <v>185</v>
+        <v>183</v>
       </c>
       <c r="G28" s="10" t="s">
-        <v>244</v>
+        <v>240</v>
       </c>
       <c r="H28" s="9" t="s">
-        <v>288</v>
+        <v>282</v>
       </c>
       <c r="I28" s="10" t="s">
-        <v>330</v>
+        <v>323</v>
       </c>
       <c r="J28" s="9">
         <v>1</v>
@@ -2712,16 +2707,16 @@
         <v>123</v>
       </c>
       <c r="F29" s="7" t="s">
-        <v>185</v>
+        <v>183</v>
       </c>
       <c r="G29" s="8" t="s">
-        <v>245</v>
+        <v>241</v>
       </c>
       <c r="H29" s="7" t="s">
-        <v>288</v>
+        <v>282</v>
       </c>
       <c r="I29" s="8" t="s">
-        <v>336</v>
+        <v>329</v>
       </c>
       <c r="J29" s="7">
         <v>1</v>
@@ -2744,16 +2739,16 @@
         <v>124</v>
       </c>
       <c r="F30" s="9" t="s">
-        <v>188</v>
+        <v>186</v>
       </c>
       <c r="G30" s="10" t="s">
-        <v>246</v>
+        <v>242</v>
       </c>
       <c r="H30" s="9" t="s">
-        <v>292</v>
+        <v>286</v>
       </c>
       <c r="I30" s="10" t="s">
-        <v>246</v>
+        <v>242</v>
       </c>
       <c r="J30" s="9">
         <v>1</v>
@@ -2767,7 +2762,7 @@
         <v>29</v>
       </c>
       <c r="C31" s="12" t="s">
-        <v>382</v>
+        <v>374</v>
       </c>
       <c r="D31" s="7" t="s">
         <v>44</v>
@@ -2776,16 +2771,16 @@
         <v>125</v>
       </c>
       <c r="F31" s="7" t="s">
-        <v>189</v>
+        <v>187</v>
       </c>
       <c r="G31" s="8" t="s">
-        <v>247</v>
+        <v>243</v>
       </c>
       <c r="H31" s="7" t="s">
-        <v>293</v>
+        <v>287</v>
       </c>
       <c r="I31" s="8" t="s">
-        <v>247</v>
+        <v>243</v>
       </c>
       <c r="J31" s="7">
         <v>1</v>
@@ -2799,7 +2794,7 @@
         <v>30</v>
       </c>
       <c r="C32" s="12" t="s">
-        <v>382</v>
+        <v>374</v>
       </c>
       <c r="D32" s="9" t="s">
         <v>45</v>
@@ -2808,14 +2803,14 @@
         <v>126</v>
       </c>
       <c r="F32" s="9" t="s">
-        <v>190</v>
+        <v>188</v>
       </c>
       <c r="G32" s="10" t="s">
-        <v>337</v>
+        <v>330</v>
       </c>
       <c r="H32" s="9"/>
       <c r="I32" s="10" t="s">
-        <v>337</v>
+        <v>330</v>
       </c>
       <c r="J32" s="9">
         <v>1</v>
@@ -2829,7 +2824,7 @@
         <v>31</v>
       </c>
       <c r="C33" s="12" t="s">
-        <v>383</v>
+        <v>375</v>
       </c>
       <c r="D33" s="7" t="s">
         <v>46</v>
@@ -2838,16 +2833,16 @@
         <v>127</v>
       </c>
       <c r="F33" s="7" t="s">
-        <v>191</v>
+        <v>189</v>
       </c>
       <c r="G33" s="8" t="s">
-        <v>191</v>
+        <v>189</v>
       </c>
       <c r="H33" s="7" t="s">
-        <v>291</v>
+        <v>285</v>
       </c>
       <c r="I33" s="8" t="s">
-        <v>191</v>
+        <v>189</v>
       </c>
       <c r="J33" s="7">
         <v>1</v>
@@ -2870,16 +2865,16 @@
         <v>128</v>
       </c>
       <c r="F34" s="9" t="s">
-        <v>192</v>
+        <v>190</v>
       </c>
       <c r="G34" s="10" t="s">
-        <v>248</v>
+        <v>244</v>
       </c>
       <c r="H34" s="9" t="s">
-        <v>291</v>
+        <v>285</v>
       </c>
       <c r="I34" s="10" t="s">
-        <v>338</v>
+        <v>331</v>
       </c>
       <c r="J34" s="9">
         <v>1</v>
@@ -2902,16 +2897,16 @@
         <v>129</v>
       </c>
       <c r="F35" s="7" t="s">
-        <v>193</v>
+        <v>191</v>
       </c>
       <c r="G35" s="8" t="s">
-        <v>249</v>
+        <v>245</v>
       </c>
       <c r="H35" s="7" t="s">
-        <v>291</v>
+        <v>285</v>
       </c>
       <c r="I35" s="8" t="s">
-        <v>249</v>
+        <v>245</v>
       </c>
       <c r="J35" s="7">
         <v>1</v>
@@ -2925,7 +2920,7 @@
         <v>34</v>
       </c>
       <c r="C36" s="13" t="s">
-        <v>384</v>
+        <v>376</v>
       </c>
       <c r="D36" s="9" t="s">
         <v>49</v>
@@ -2934,14 +2929,14 @@
         <v>130</v>
       </c>
       <c r="F36" s="9" t="s">
-        <v>194</v>
+        <v>192</v>
       </c>
       <c r="G36" s="10" t="s">
-        <v>339</v>
+        <v>332</v>
       </c>
       <c r="H36" s="9"/>
       <c r="I36" s="10" t="s">
-        <v>339</v>
+        <v>332</v>
       </c>
       <c r="J36" s="9">
         <v>1</v>
@@ -2955,7 +2950,7 @@
         <v>35</v>
       </c>
       <c r="C37" s="13" t="s">
-        <v>384</v>
+        <v>376</v>
       </c>
       <c r="D37" s="7" t="s">
         <v>50</v>
@@ -2964,14 +2959,14 @@
         <v>131</v>
       </c>
       <c r="F37" s="7" t="s">
-        <v>195</v>
+        <v>193</v>
       </c>
       <c r="G37" s="8" t="s">
-        <v>340</v>
+        <v>333</v>
       </c>
       <c r="H37" s="7"/>
       <c r="I37" s="8" t="s">
-        <v>340</v>
+        <v>333</v>
       </c>
       <c r="J37" s="7">
         <v>1</v>
@@ -2985,7 +2980,7 @@
         <v>36</v>
       </c>
       <c r="C38" s="13" t="s">
-        <v>403</v>
+        <v>395</v>
       </c>
       <c r="D38" s="9" t="s">
         <v>51</v>
@@ -2994,23 +2989,23 @@
         <v>132</v>
       </c>
       <c r="F38" s="9" t="s">
-        <v>196</v>
+        <v>194</v>
       </c>
       <c r="G38" s="10" t="s">
-        <v>402</v>
+        <v>394</v>
       </c>
       <c r="H38" s="9" t="s">
-        <v>404</v>
+        <v>396</v>
       </c>
       <c r="I38" s="10" t="s">
-        <v>341</v>
+        <v>334</v>
       </c>
       <c r="J38" s="9">
         <v>1</v>
       </c>
       <c r="K38" s="9"/>
     </row>
-    <row r="39" spans="1:11" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="39" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A39" s="1"/>
       <c r="B39" s="11">
         <f>ROW(B39) - ROW($B$2)</f>
@@ -3023,19 +3018,19 @@
         <v>52</v>
       </c>
       <c r="E39" s="8" t="s">
-        <v>133</v>
-      </c>
-      <c r="F39" s="7" t="s">
-        <v>197</v>
+        <v>414</v>
+      </c>
+      <c r="F39" s="7">
+        <v>2036150003</v>
       </c>
       <c r="G39" s="8" t="s">
-        <v>250</v>
+        <v>415</v>
       </c>
       <c r="H39" s="7" t="s">
-        <v>294</v>
+        <v>416</v>
       </c>
       <c r="I39" s="8" t="s">
-        <v>250</v>
+        <v>415</v>
       </c>
       <c r="J39" s="7">
         <v>1</v>
@@ -3049,25 +3044,25 @@
         <v>38</v>
       </c>
       <c r="C40" s="13" t="s">
-        <v>385</v>
+        <v>377</v>
       </c>
       <c r="D40" s="9" t="s">
         <v>53</v>
       </c>
       <c r="E40" s="10" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="F40" s="9" t="s">
-        <v>198</v>
+        <v>195</v>
       </c>
       <c r="G40" s="10" t="s">
-        <v>251</v>
+        <v>246</v>
       </c>
       <c r="H40" s="9" t="s">
-        <v>295</v>
+        <v>289</v>
       </c>
       <c r="I40" s="10" t="s">
-        <v>251</v>
+        <v>246</v>
       </c>
       <c r="J40" s="9">
         <v>1</v>
@@ -3087,19 +3082,19 @@
         <v>54</v>
       </c>
       <c r="E41" s="8" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="F41" s="7" t="s">
-        <v>199</v>
+        <v>196</v>
       </c>
       <c r="G41" s="8" t="s">
-        <v>405</v>
+        <v>397</v>
       </c>
       <c r="H41" s="7" t="s">
-        <v>390</v>
+        <v>382</v>
       </c>
       <c r="I41" s="8" t="s">
-        <v>342</v>
+        <v>335</v>
       </c>
       <c r="J41" s="7">
         <v>1</v>
@@ -3119,19 +3114,19 @@
         <v>55</v>
       </c>
       <c r="E42" s="10" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="F42" s="9" t="s">
-        <v>200</v>
+        <v>197</v>
       </c>
       <c r="G42" s="10" t="s">
-        <v>406</v>
+        <v>398</v>
       </c>
       <c r="H42" s="7" t="s">
-        <v>390</v>
+        <v>382</v>
       </c>
       <c r="I42" s="10" t="s">
-        <v>343</v>
+        <v>336</v>
       </c>
       <c r="J42" s="9">
         <v>1</v>
@@ -3147,29 +3142,29 @@
       <c r="C43" s="12" t="s">
         <v>7</v>
       </c>
-      <c r="D43" s="15" t="s">
+      <c r="D43" s="14" t="s">
         <v>56</v>
       </c>
-      <c r="E43" s="16" t="s">
-        <v>136</v>
-      </c>
-      <c r="F43" s="15" t="s">
-        <v>200</v>
-      </c>
-      <c r="G43" s="16" t="s">
-        <v>401</v>
-      </c>
-      <c r="H43" s="15" t="s">
-        <v>401</v>
-      </c>
-      <c r="I43" s="16" t="s">
-        <v>333</v>
-      </c>
-      <c r="J43" s="15">
-        <v>1</v>
-      </c>
-      <c r="K43" s="17" t="s">
-        <v>381</v>
+      <c r="E43" s="15" t="s">
+        <v>135</v>
+      </c>
+      <c r="F43" s="14" t="s">
+        <v>197</v>
+      </c>
+      <c r="G43" s="15" t="s">
+        <v>393</v>
+      </c>
+      <c r="H43" s="14" t="s">
+        <v>393</v>
+      </c>
+      <c r="I43" s="15" t="s">
+        <v>326</v>
+      </c>
+      <c r="J43" s="14">
+        <v>1</v>
+      </c>
+      <c r="K43" s="16" t="s">
+        <v>373</v>
       </c>
     </row>
     <row r="44" spans="1:11" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
@@ -3185,19 +3180,19 @@
         <v>57</v>
       </c>
       <c r="E44" s="10" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="F44" s="9" t="s">
-        <v>200</v>
+        <v>197</v>
       </c>
       <c r="G44" s="10" t="s">
-        <v>407</v>
+        <v>399</v>
       </c>
       <c r="H44" s="9" t="s">
-        <v>408</v>
+        <v>400</v>
       </c>
       <c r="I44" s="10" t="s">
-        <v>344</v>
+        <v>337</v>
       </c>
       <c r="J44" s="9">
         <v>1</v>
@@ -3217,19 +3212,19 @@
         <v>58</v>
       </c>
       <c r="E45" s="8" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="F45" s="7" t="s">
-        <v>200</v>
+        <v>197</v>
       </c>
       <c r="G45" s="8" t="s">
-        <v>409</v>
+        <v>401</v>
       </c>
       <c r="H45" s="7" t="s">
-        <v>390</v>
+        <v>382</v>
       </c>
       <c r="I45" s="8" t="s">
-        <v>345</v>
+        <v>338</v>
       </c>
       <c r="J45" s="7">
         <v>2</v>
@@ -3249,19 +3244,19 @@
         <v>59</v>
       </c>
       <c r="E46" s="10" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="F46" s="9" t="s">
-        <v>199</v>
+        <v>196</v>
       </c>
       <c r="G46" s="10" t="s">
-        <v>252</v>
+        <v>247</v>
       </c>
       <c r="H46" s="9" t="s">
-        <v>291</v>
+        <v>285</v>
       </c>
       <c r="I46" s="10" t="s">
-        <v>346</v>
+        <v>339</v>
       </c>
       <c r="J46" s="9">
         <v>1</v>
@@ -3281,19 +3276,19 @@
         <v>60</v>
       </c>
       <c r="E47" s="8" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="F47" s="7" t="s">
-        <v>201</v>
+        <v>198</v>
       </c>
       <c r="G47" s="8" t="s">
-        <v>410</v>
+        <v>402</v>
       </c>
       <c r="H47" s="7" t="s">
-        <v>390</v>
+        <v>382</v>
       </c>
       <c r="I47" s="8" t="s">
-        <v>347</v>
+        <v>340</v>
       </c>
       <c r="J47" s="7">
         <v>1</v>
@@ -3313,19 +3308,19 @@
         <v>61</v>
       </c>
       <c r="E48" s="10" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="F48" s="9" t="s">
-        <v>202</v>
+        <v>199</v>
       </c>
       <c r="G48" s="10" t="s">
-        <v>411</v>
+        <v>403</v>
       </c>
       <c r="H48" s="7" t="s">
-        <v>390</v>
+        <v>382</v>
       </c>
       <c r="I48" s="10" t="s">
-        <v>348</v>
+        <v>341</v>
       </c>
       <c r="J48" s="9">
         <v>1</v>
@@ -3345,19 +3340,19 @@
         <v>62</v>
       </c>
       <c r="E49" s="8" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="F49" s="7" t="s">
-        <v>203</v>
+        <v>200</v>
       </c>
       <c r="G49" s="8" t="s">
-        <v>412</v>
+        <v>404</v>
       </c>
       <c r="H49" s="7" t="s">
-        <v>390</v>
+        <v>382</v>
       </c>
       <c r="I49" s="8" t="s">
-        <v>349</v>
+        <v>342</v>
       </c>
       <c r="J49" s="7">
         <v>1</v>
@@ -3377,19 +3372,19 @@
         <v>63</v>
       </c>
       <c r="E50" s="10" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="F50" s="9" t="s">
-        <v>204</v>
+        <v>201</v>
       </c>
       <c r="G50" s="10" t="s">
-        <v>204</v>
+        <v>201</v>
       </c>
       <c r="H50" s="9" t="s">
-        <v>296</v>
+        <v>290</v>
       </c>
       <c r="I50" s="10" t="s">
-        <v>350</v>
+        <v>343</v>
       </c>
       <c r="J50" s="9">
         <v>1</v>
@@ -3409,19 +3404,19 @@
         <v>64</v>
       </c>
       <c r="E51" s="8" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="F51" s="7" t="s">
-        <v>205</v>
+        <v>202</v>
       </c>
       <c r="G51" s="8" t="s">
-        <v>253</v>
+        <v>248</v>
       </c>
       <c r="H51" s="7" t="s">
-        <v>297</v>
+        <v>291</v>
       </c>
       <c r="I51" s="8" t="s">
-        <v>351</v>
+        <v>344</v>
       </c>
       <c r="J51" s="7">
         <v>1</v>
@@ -3441,19 +3436,19 @@
         <v>65</v>
       </c>
       <c r="E52" s="10" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="F52" s="9" t="s">
-        <v>200</v>
+        <v>197</v>
       </c>
       <c r="G52" s="10" t="s">
-        <v>254</v>
+        <v>249</v>
       </c>
       <c r="H52" s="9" t="s">
-        <v>291</v>
+        <v>285</v>
       </c>
       <c r="I52" s="10" t="s">
-        <v>352</v>
+        <v>345</v>
       </c>
       <c r="J52" s="9">
         <v>1</v>
@@ -3473,19 +3468,19 @@
         <v>66</v>
       </c>
       <c r="E53" s="8" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="F53" s="7" t="s">
-        <v>206</v>
+        <v>203</v>
       </c>
       <c r="G53" s="8" t="s">
-        <v>255</v>
+        <v>250</v>
       </c>
       <c r="H53" s="7" t="s">
-        <v>291</v>
+        <v>285</v>
       </c>
       <c r="I53" s="8" t="s">
-        <v>342</v>
+        <v>335</v>
       </c>
       <c r="J53" s="7">
         <v>1</v>
@@ -3505,19 +3500,19 @@
         <v>67</v>
       </c>
       <c r="E54" s="10" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="F54" s="9" t="s">
-        <v>207</v>
+        <v>204</v>
       </c>
       <c r="G54" s="10" t="s">
-        <v>256</v>
+        <v>251</v>
       </c>
       <c r="H54" s="9" t="s">
-        <v>289</v>
+        <v>283</v>
       </c>
       <c r="I54" s="10" t="s">
-        <v>353</v>
+        <v>346</v>
       </c>
       <c r="J54" s="9">
         <v>1</v>
@@ -3538,16 +3533,16 @@
       </c>
       <c r="E55" s="8"/>
       <c r="F55" s="7" t="s">
-        <v>208</v>
+        <v>205</v>
       </c>
       <c r="G55" s="8" t="s">
-        <v>413</v>
+        <v>405</v>
       </c>
       <c r="H55" s="7" t="s">
-        <v>414</v>
+        <v>406</v>
       </c>
       <c r="I55" s="8" t="s">
-        <v>354</v>
+        <v>347</v>
       </c>
       <c r="J55" s="7">
         <v>1</v>
@@ -3567,19 +3562,19 @@
         <v>69</v>
       </c>
       <c r="E56" s="10" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="F56" s="9" t="s">
-        <v>209</v>
+        <v>206</v>
       </c>
       <c r="G56" s="10" t="s">
-        <v>257</v>
+        <v>252</v>
       </c>
       <c r="H56" s="9" t="s">
-        <v>298</v>
+        <v>292</v>
       </c>
       <c r="I56" s="10" t="s">
-        <v>355</v>
+        <v>348</v>
       </c>
       <c r="J56" s="9">
         <v>1</v>
@@ -3599,53 +3594,53 @@
         <v>70</v>
       </c>
       <c r="E57" s="8" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="F57" s="7" t="s">
-        <v>209</v>
+        <v>206</v>
       </c>
       <c r="G57" s="8" t="s">
-        <v>258</v>
+        <v>253</v>
       </c>
       <c r="H57" s="7" t="s">
-        <v>298</v>
+        <v>292</v>
       </c>
       <c r="I57" s="8" t="s">
-        <v>356</v>
+        <v>349</v>
       </c>
       <c r="J57" s="7">
         <v>1</v>
       </c>
       <c r="K57" s="7"/>
     </row>
-    <row r="58" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="58" spans="1:11" ht="36.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A58" s="1"/>
       <c r="B58" s="11">
         <f t="shared" si="0"/>
         <v>56</v>
       </c>
       <c r="C58" s="13" t="s">
-        <v>386</v>
+        <v>378</v>
       </c>
       <c r="D58" s="9" t="s">
         <v>71</v>
       </c>
-      <c r="E58" s="10" t="s">
-        <v>147</v>
-      </c>
-      <c r="F58" s="9" t="s">
-        <v>210</v>
-      </c>
-      <c r="G58" s="10" t="s">
-        <v>259</v>
-      </c>
-      <c r="H58" s="9" t="s">
-        <v>299</v>
-      </c>
-      <c r="I58" s="10" t="s">
-        <v>357</v>
-      </c>
-      <c r="J58" s="9">
+      <c r="E58" s="8" t="s">
+        <v>417</v>
+      </c>
+      <c r="F58" s="7" t="s">
+        <v>418</v>
+      </c>
+      <c r="G58" s="8" t="s">
+        <v>418</v>
+      </c>
+      <c r="H58" s="7" t="s">
+        <v>419</v>
+      </c>
+      <c r="I58" s="8" t="s">
+        <v>418</v>
+      </c>
+      <c r="J58" s="7">
         <v>1</v>
       </c>
       <c r="K58" s="9"/>
@@ -3657,25 +3652,25 @@
         <v>57</v>
       </c>
       <c r="C59" s="12" t="s">
-        <v>387</v>
+        <v>379</v>
       </c>
       <c r="D59" s="7" t="s">
         <v>72</v>
       </c>
       <c r="E59" s="8" t="s">
-        <v>148</v>
+        <v>146</v>
       </c>
       <c r="F59" s="7" t="s">
-        <v>211</v>
+        <v>207</v>
       </c>
       <c r="G59" s="8" t="s">
-        <v>358</v>
+        <v>350</v>
       </c>
       <c r="H59" s="7" t="s">
-        <v>415</v>
+        <v>407</v>
       </c>
       <c r="I59" s="8" t="s">
-        <v>358</v>
+        <v>350</v>
       </c>
       <c r="J59" s="7">
         <v>3</v>
@@ -3689,25 +3684,25 @@
         <v>58</v>
       </c>
       <c r="C60" s="12" t="s">
-        <v>387</v>
+        <v>379</v>
       </c>
       <c r="D60" s="9" t="s">
         <v>73</v>
       </c>
       <c r="E60" s="10" t="s">
-        <v>149</v>
+        <v>147</v>
       </c>
       <c r="F60" s="9" t="s">
-        <v>211</v>
+        <v>207</v>
       </c>
       <c r="G60" s="10" t="s">
-        <v>416</v>
+        <v>408</v>
       </c>
       <c r="H60" s="9" t="s">
-        <v>417</v>
+        <v>409</v>
       </c>
       <c r="I60" s="10" t="s">
-        <v>359</v>
+        <v>351</v>
       </c>
       <c r="J60" s="9">
         <v>1</v>
@@ -3727,19 +3722,19 @@
         <v>74</v>
       </c>
       <c r="E61" s="8" t="s">
-        <v>150</v>
+        <v>148</v>
       </c>
       <c r="F61" s="7" t="s">
-        <v>212</v>
+        <v>208</v>
       </c>
       <c r="G61" s="8" t="s">
-        <v>260</v>
+        <v>254</v>
       </c>
       <c r="H61" s="7" t="s">
-        <v>288</v>
+        <v>282</v>
       </c>
       <c r="I61" s="8" t="s">
-        <v>360</v>
+        <v>352</v>
       </c>
       <c r="J61" s="7">
         <v>2</v>
@@ -3759,19 +3754,19 @@
         <v>75</v>
       </c>
       <c r="E62" s="10" t="s">
-        <v>151</v>
+        <v>149</v>
       </c>
       <c r="F62" s="9" t="s">
-        <v>213</v>
+        <v>209</v>
       </c>
       <c r="G62" s="10" t="s">
-        <v>261</v>
+        <v>255</v>
       </c>
       <c r="H62" s="9" t="s">
-        <v>288</v>
+        <v>282</v>
       </c>
       <c r="I62" s="10" t="s">
-        <v>361</v>
+        <v>353</v>
       </c>
       <c r="J62" s="9">
         <v>3</v>
@@ -3791,19 +3786,19 @@
         <v>76</v>
       </c>
       <c r="E63" s="8" t="s">
-        <v>152</v>
+        <v>150</v>
       </c>
       <c r="F63" s="7" t="s">
-        <v>213</v>
+        <v>209</v>
       </c>
       <c r="G63" s="8" t="s">
-        <v>262</v>
+        <v>256</v>
       </c>
       <c r="H63" s="7" t="s">
-        <v>288</v>
+        <v>282</v>
       </c>
       <c r="I63" s="8" t="s">
-        <v>362</v>
+        <v>354</v>
       </c>
       <c r="J63" s="7">
         <v>8</v>
@@ -3823,19 +3818,19 @@
         <v>77</v>
       </c>
       <c r="E64" s="10" t="s">
-        <v>153</v>
+        <v>151</v>
       </c>
       <c r="F64" s="9" t="s">
-        <v>213</v>
+        <v>209</v>
       </c>
       <c r="G64" s="10" t="s">
-        <v>263</v>
+        <v>257</v>
       </c>
       <c r="H64" s="9" t="s">
-        <v>288</v>
+        <v>282</v>
       </c>
       <c r="I64" s="10" t="s">
-        <v>363</v>
+        <v>355</v>
       </c>
       <c r="J64" s="9">
         <v>5</v>
@@ -3855,19 +3850,19 @@
         <v>78</v>
       </c>
       <c r="E65" s="8" t="s">
-        <v>154</v>
+        <v>152</v>
       </c>
       <c r="F65" s="7" t="s">
-        <v>213</v>
+        <v>209</v>
       </c>
       <c r="G65" s="8" t="s">
-        <v>264</v>
+        <v>258</v>
       </c>
       <c r="H65" s="7" t="s">
-        <v>288</v>
+        <v>282</v>
       </c>
       <c r="I65" s="8" t="s">
-        <v>364</v>
+        <v>356</v>
       </c>
       <c r="J65" s="7">
         <v>3</v>
@@ -3883,29 +3878,29 @@
       <c r="C66" s="13" t="s">
         <v>11</v>
       </c>
-      <c r="D66" s="15" t="s">
+      <c r="D66" s="14" t="s">
         <v>79</v>
       </c>
-      <c r="E66" s="16" t="s">
-        <v>155</v>
-      </c>
-      <c r="F66" s="15" t="s">
-        <v>213</v>
-      </c>
-      <c r="G66" s="16" t="s">
-        <v>265</v>
-      </c>
-      <c r="H66" s="15" t="s">
-        <v>288</v>
-      </c>
-      <c r="I66" s="16" t="s">
-        <v>333</v>
-      </c>
-      <c r="J66" s="15">
+      <c r="E66" s="15" t="s">
+        <v>153</v>
+      </c>
+      <c r="F66" s="14" t="s">
+        <v>209</v>
+      </c>
+      <c r="G66" s="15" t="s">
+        <v>259</v>
+      </c>
+      <c r="H66" s="14" t="s">
+        <v>282</v>
+      </c>
+      <c r="I66" s="15" t="s">
+        <v>326</v>
+      </c>
+      <c r="J66" s="14">
         <v>9</v>
       </c>
-      <c r="K66" s="17" t="s">
-        <v>381</v>
+      <c r="K66" s="16" t="s">
+        <v>373</v>
       </c>
     </row>
     <row r="67" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
@@ -3921,19 +3916,19 @@
         <v>80</v>
       </c>
       <c r="E67" s="8" t="s">
-        <v>156</v>
+        <v>154</v>
       </c>
       <c r="F67" s="7" t="s">
-        <v>213</v>
+        <v>209</v>
       </c>
       <c r="G67" s="8" t="s">
-        <v>266</v>
+        <v>260</v>
       </c>
       <c r="H67" s="7" t="s">
-        <v>288</v>
+        <v>282</v>
       </c>
       <c r="I67" s="8" t="s">
-        <v>365</v>
+        <v>357</v>
       </c>
       <c r="J67" s="7">
         <v>1</v>
@@ -3953,19 +3948,19 @@
         <v>81</v>
       </c>
       <c r="E68" s="10" t="s">
-        <v>157</v>
+        <v>155</v>
       </c>
       <c r="F68" s="9" t="s">
-        <v>213</v>
+        <v>209</v>
       </c>
       <c r="G68" s="10" t="s">
-        <v>267</v>
+        <v>261</v>
       </c>
       <c r="H68" s="9" t="s">
-        <v>288</v>
+        <v>282</v>
       </c>
       <c r="I68" s="10" t="s">
-        <v>366</v>
+        <v>358</v>
       </c>
       <c r="J68" s="9">
         <v>2</v>
@@ -3985,19 +3980,19 @@
         <v>82</v>
       </c>
       <c r="E69" s="8" t="s">
-        <v>155</v>
+        <v>153</v>
       </c>
       <c r="F69" s="7" t="s">
-        <v>213</v>
+        <v>209</v>
       </c>
       <c r="G69" s="8" t="s">
-        <v>265</v>
+        <v>259</v>
       </c>
       <c r="H69" s="7" t="s">
-        <v>288</v>
+        <v>282</v>
       </c>
       <c r="I69" s="8" t="s">
-        <v>360</v>
+        <v>352</v>
       </c>
       <c r="J69" s="7">
         <v>3</v>
@@ -4017,19 +4012,19 @@
         <v>83</v>
       </c>
       <c r="E70" s="10" t="s">
-        <v>158</v>
+        <v>156</v>
       </c>
       <c r="F70" s="9" t="s">
-        <v>213</v>
+        <v>209</v>
       </c>
       <c r="G70" s="10" t="s">
-        <v>268</v>
+        <v>262</v>
       </c>
       <c r="H70" s="9" t="s">
-        <v>288</v>
+        <v>282</v>
       </c>
       <c r="I70" s="10" t="s">
-        <v>367</v>
+        <v>359</v>
       </c>
       <c r="J70" s="9">
         <v>2</v>
@@ -4049,19 +4044,19 @@
         <v>84</v>
       </c>
       <c r="E71" s="8" t="s">
-        <v>159</v>
+        <v>157</v>
       </c>
       <c r="F71" s="7" t="s">
-        <v>213</v>
+        <v>209</v>
       </c>
       <c r="G71" s="8" t="s">
-        <v>269</v>
+        <v>263</v>
       </c>
       <c r="H71" s="7" t="s">
-        <v>300</v>
+        <v>293</v>
       </c>
       <c r="I71" s="8" t="s">
-        <v>368</v>
+        <v>360</v>
       </c>
       <c r="J71" s="7">
         <v>1</v>
@@ -4081,19 +4076,19 @@
         <v>85</v>
       </c>
       <c r="E72" s="10" t="s">
-        <v>160</v>
+        <v>158</v>
       </c>
       <c r="F72" s="9" t="s">
-        <v>214</v>
+        <v>210</v>
       </c>
       <c r="G72" s="10" t="s">
-        <v>270</v>
+        <v>264</v>
       </c>
       <c r="H72" s="9" t="s">
-        <v>288</v>
+        <v>282</v>
       </c>
       <c r="I72" s="10" t="s">
-        <v>363</v>
+        <v>355</v>
       </c>
       <c r="J72" s="9">
         <v>1</v>
@@ -4113,19 +4108,19 @@
         <v>86</v>
       </c>
       <c r="E73" s="8" t="s">
-        <v>161</v>
+        <v>159</v>
       </c>
       <c r="F73" s="7" t="s">
-        <v>215</v>
+        <v>211</v>
       </c>
       <c r="G73" s="8" t="s">
-        <v>271</v>
+        <v>265</v>
       </c>
       <c r="H73" s="7" t="s">
-        <v>301</v>
+        <v>294</v>
       </c>
       <c r="I73" s="8" t="s">
-        <v>369</v>
+        <v>361</v>
       </c>
       <c r="J73" s="7">
         <v>1</v>
@@ -4145,19 +4140,19 @@
         <v>87</v>
       </c>
       <c r="E74" s="10" t="s">
-        <v>162</v>
+        <v>160</v>
       </c>
       <c r="F74" s="9" t="s">
-        <v>215</v>
+        <v>211</v>
       </c>
       <c r="G74" s="10" t="s">
-        <v>272</v>
+        <v>266</v>
       </c>
       <c r="H74" s="9" t="s">
-        <v>288</v>
+        <v>282</v>
       </c>
       <c r="I74" s="10" t="s">
-        <v>370</v>
+        <v>362</v>
       </c>
       <c r="J74" s="9">
         <v>1</v>
@@ -4177,19 +4172,19 @@
         <v>88</v>
       </c>
       <c r="E75" s="8" t="s">
-        <v>163</v>
+        <v>161</v>
       </c>
       <c r="F75" s="7" t="s">
-        <v>213</v>
+        <v>209</v>
       </c>
       <c r="G75" s="8" t="s">
-        <v>273</v>
+        <v>267</v>
       </c>
       <c r="H75" s="7" t="s">
-        <v>288</v>
+        <v>282</v>
       </c>
       <c r="I75" s="8" t="s">
-        <v>371</v>
+        <v>363</v>
       </c>
       <c r="J75" s="7">
         <v>2</v>
@@ -4203,25 +4198,25 @@
         <v>74</v>
       </c>
       <c r="C76" s="13" t="s">
-        <v>388</v>
+        <v>380</v>
       </c>
       <c r="D76" s="9" t="s">
         <v>89</v>
       </c>
       <c r="E76" s="10" t="s">
-        <v>164</v>
+        <v>162</v>
       </c>
       <c r="F76" s="9" t="s">
-        <v>216</v>
+        <v>212</v>
       </c>
       <c r="G76" s="10" t="s">
-        <v>216</v>
+        <v>212</v>
       </c>
       <c r="H76" s="9" t="s">
-        <v>294</v>
+        <v>288</v>
       </c>
       <c r="I76" s="10" t="s">
-        <v>216</v>
+        <v>212</v>
       </c>
       <c r="J76" s="9">
         <v>1</v>
@@ -4241,19 +4236,19 @@
         <v>90</v>
       </c>
       <c r="E77" s="8" t="s">
-        <v>165</v>
+        <v>163</v>
       </c>
       <c r="F77" s="7" t="s">
-        <v>217</v>
+        <v>213</v>
       </c>
       <c r="G77" s="8" t="s">
-        <v>372</v>
+        <v>364</v>
       </c>
       <c r="H77" s="7" t="s">
-        <v>418</v>
+        <v>410</v>
       </c>
       <c r="I77" s="8" t="s">
-        <v>372</v>
+        <v>364</v>
       </c>
       <c r="J77" s="7">
         <v>2</v>
@@ -4273,19 +4268,19 @@
         <v>91</v>
       </c>
       <c r="E78" s="10" t="s">
-        <v>166</v>
+        <v>164</v>
       </c>
       <c r="F78" s="9" t="s">
-        <v>218</v>
+        <v>214</v>
       </c>
       <c r="G78" s="10" t="s">
-        <v>274</v>
+        <v>268</v>
       </c>
       <c r="H78" s="9" t="s">
-        <v>302</v>
+        <v>295</v>
       </c>
       <c r="I78" s="10" t="s">
-        <v>373</v>
+        <v>365</v>
       </c>
       <c r="J78" s="9">
         <v>1</v>
@@ -4305,19 +4300,19 @@
         <v>92</v>
       </c>
       <c r="E79" s="8" t="s">
-        <v>167</v>
+        <v>165</v>
       </c>
       <c r="F79" s="7" t="s">
-        <v>219</v>
+        <v>215</v>
       </c>
       <c r="G79" s="8" t="s">
-        <v>275</v>
+        <v>269</v>
       </c>
       <c r="H79" s="7" t="s">
-        <v>303</v>
+        <v>296</v>
       </c>
       <c r="I79" s="8" t="s">
-        <v>275</v>
+        <v>269</v>
       </c>
       <c r="J79" s="7">
         <v>1</v>
@@ -4337,19 +4332,19 @@
         <v>93</v>
       </c>
       <c r="E80" s="10" t="s">
-        <v>168</v>
+        <v>166</v>
       </c>
       <c r="F80" s="9" t="s">
-        <v>220</v>
+        <v>216</v>
       </c>
       <c r="G80" s="10" t="s">
-        <v>276</v>
+        <v>270</v>
       </c>
       <c r="H80" s="9" t="s">
-        <v>304</v>
+        <v>297</v>
       </c>
       <c r="I80" s="10" t="s">
-        <v>276</v>
+        <v>270</v>
       </c>
       <c r="J80" s="9">
         <v>1</v>
@@ -4369,19 +4364,19 @@
         <v>94</v>
       </c>
       <c r="E81" s="8" t="s">
-        <v>169</v>
+        <v>167</v>
       </c>
       <c r="F81" s="7" t="s">
-        <v>221</v>
+        <v>217</v>
       </c>
       <c r="G81" s="8" t="s">
-        <v>277</v>
+        <v>271</v>
       </c>
       <c r="H81" s="7" t="s">
-        <v>305</v>
+        <v>298</v>
       </c>
       <c r="I81" s="8" t="s">
-        <v>277</v>
+        <v>271</v>
       </c>
       <c r="J81" s="7">
         <v>1</v>
@@ -4401,17 +4396,17 @@
         <v>95</v>
       </c>
       <c r="E82" s="10" t="s">
-        <v>170</v>
+        <v>168</v>
       </c>
       <c r="F82" s="9" t="s">
-        <v>222</v>
+        <v>218</v>
       </c>
       <c r="G82" s="10" t="s">
-        <v>374</v>
+        <v>366</v>
       </c>
       <c r="H82" s="9"/>
       <c r="I82" s="10" t="s">
-        <v>374</v>
+        <v>366</v>
       </c>
       <c r="J82" s="9">
         <v>1</v>
@@ -4431,19 +4426,19 @@
         <v>96</v>
       </c>
       <c r="E83" s="8" t="s">
-        <v>171</v>
+        <v>169</v>
       </c>
       <c r="F83" s="7" t="s">
-        <v>223</v>
+        <v>219</v>
       </c>
       <c r="G83" s="8" t="s">
-        <v>278</v>
+        <v>272</v>
       </c>
       <c r="H83" s="7" t="s">
-        <v>306</v>
+        <v>299</v>
       </c>
       <c r="I83" s="8" t="s">
-        <v>278</v>
+        <v>272</v>
       </c>
       <c r="J83" s="7">
         <v>1</v>
@@ -4463,19 +4458,19 @@
         <v>97</v>
       </c>
       <c r="E84" s="10" t="s">
-        <v>172</v>
+        <v>170</v>
       </c>
       <c r="F84" s="9" t="s">
-        <v>224</v>
+        <v>220</v>
       </c>
       <c r="G84" s="10" t="s">
-        <v>279</v>
+        <v>273</v>
       </c>
       <c r="H84" s="9" t="s">
-        <v>307</v>
+        <v>300</v>
       </c>
       <c r="I84" s="10" t="s">
-        <v>375</v>
+        <v>367</v>
       </c>
       <c r="J84" s="9">
         <v>1</v>
@@ -4495,19 +4490,19 @@
         <v>98</v>
       </c>
       <c r="E85" s="8" t="s">
-        <v>173</v>
+        <v>171</v>
       </c>
       <c r="F85" s="7" t="s">
-        <v>225</v>
+        <v>221</v>
       </c>
       <c r="G85" s="8" t="s">
-        <v>280</v>
+        <v>274</v>
       </c>
       <c r="H85" s="7" t="s">
-        <v>308</v>
+        <v>301</v>
       </c>
       <c r="I85" s="8" t="s">
-        <v>280</v>
+        <v>274</v>
       </c>
       <c r="J85" s="7">
         <v>1</v>
@@ -4527,19 +4522,19 @@
         <v>99</v>
       </c>
       <c r="E86" s="10" t="s">
-        <v>174</v>
+        <v>172</v>
       </c>
       <c r="F86" s="9" t="s">
-        <v>226</v>
+        <v>222</v>
       </c>
       <c r="G86" s="10" t="s">
-        <v>281</v>
+        <v>275</v>
       </c>
       <c r="H86" s="9" t="s">
-        <v>293</v>
+        <v>287</v>
       </c>
       <c r="I86" s="10" t="s">
-        <v>281</v>
+        <v>275</v>
       </c>
       <c r="J86" s="9">
         <v>1</v>
@@ -4559,19 +4554,19 @@
         <v>100</v>
       </c>
       <c r="E87" s="8" t="s">
-        <v>175</v>
+        <v>173</v>
       </c>
       <c r="F87" s="7" t="s">
-        <v>227</v>
+        <v>223</v>
       </c>
       <c r="G87" s="8" t="s">
-        <v>282</v>
+        <v>276</v>
       </c>
       <c r="H87" s="7" t="s">
-        <v>309</v>
+        <v>302</v>
       </c>
       <c r="I87" s="8" t="s">
-        <v>282</v>
+        <v>276</v>
       </c>
       <c r="J87" s="7">
         <v>1</v>
@@ -4591,19 +4586,19 @@
         <v>101</v>
       </c>
       <c r="E88" s="10" t="s">
-        <v>176</v>
+        <v>174</v>
       </c>
       <c r="F88" s="9" t="s">
-        <v>228</v>
+        <v>224</v>
       </c>
       <c r="G88" s="10" t="s">
-        <v>283</v>
+        <v>277</v>
       </c>
       <c r="H88" s="9" t="s">
-        <v>310</v>
+        <v>303</v>
       </c>
       <c r="I88" s="10" t="s">
-        <v>283</v>
+        <v>277</v>
       </c>
       <c r="J88" s="9">
         <v>1</v>
@@ -4623,19 +4618,19 @@
         <v>102</v>
       </c>
       <c r="E89" s="8" t="s">
-        <v>177</v>
+        <v>175</v>
       </c>
       <c r="F89" s="7" t="s">
-        <v>229</v>
+        <v>225</v>
       </c>
       <c r="G89" s="8" t="s">
-        <v>419</v>
+        <v>411</v>
       </c>
       <c r="H89" s="7" t="s">
-        <v>420</v>
+        <v>412</v>
       </c>
       <c r="I89" s="8" t="s">
-        <v>376</v>
+        <v>368</v>
       </c>
       <c r="J89" s="7">
         <v>1</v>
@@ -4655,19 +4650,19 @@
         <v>103</v>
       </c>
       <c r="E90" s="10" t="s">
-        <v>178</v>
+        <v>176</v>
       </c>
       <c r="F90" s="9" t="s">
-        <v>230</v>
+        <v>226</v>
       </c>
       <c r="G90" s="10" t="s">
-        <v>284</v>
+        <v>278</v>
       </c>
       <c r="H90" s="9" t="s">
-        <v>311</v>
+        <v>304</v>
       </c>
       <c r="I90" s="10" t="s">
-        <v>377</v>
+        <v>369</v>
       </c>
       <c r="J90" s="9">
         <v>1</v>

</xml_diff>